<commit_message>
L08 tutorial: OpenAlex as open baseline, abstract retrieval, WoS digression
- Steps 3-6 rewritten for OpenAlex (syntax, web interface, recall test
  with closed-access papers, compulsory snowballing)
- New sub-step for filling in missing abstracts (publisher page via DOI,
  open-access versions, Crossref)
- Web of Science as a single digression: what it adds, what it costs,
  comparison exercise
- R part now queries OpenAlex directly with openalexR (API key kept in
  .Renviron), measures the abstract gap, snowballs with oa_snowball(),
  fills abstracts from Crossref, compares with a WoS export by DOI
- Templates: search log and screening sheet adapted (query URL,
  abstract source)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JpaXNUFc4pCZDmX3yDuiZt
</commit_message>
<xml_diff>
--- a/content/lecture/lit-review-tutorial/L08-review-templates.xlsx
+++ b/content/lecture/lit-review-tutorial/L08-review-templates.xlsx
@@ -483,7 +483,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Screening — one row per record from the database export (or let R build it, see the tutorial).</t>
+          <t>Screening — one row per record from the OpenAlex export (or let R build it, see the tutorial). Fill in missing abstracts first.</t>
         </is>
       </c>
     </row>
@@ -522,18 +522,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -544,7 +546,7 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Database and indexes</t>
+          <t>Database and route</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
@@ -559,25 +561,35 @@
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
+          <t>Search field</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
           <t>Filters</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Results before filters</t>
-        </is>
-      </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Results after filters</t>
+          <t>Results</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
+          <t>Query URL or script</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
           <t>Test set found (x of n)</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Share without abstract</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Change from previous version / notes</t>
         </is>
@@ -591,7 +603,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Web of Science Core Collection</t>
+          <t>OpenAlex, web interface</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -601,24 +613,34 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>TS=("four-day week*" OR "working time reduction") AND TS=(productiv* OR well-being)</t>
+          <t>("four-day week" OR "working time reduction") AND (productivity OR "well-being")</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Document types: Article, Review; Language: English</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="n"/>
+          <t>Title and abstract</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Type: article, review; language: English</t>
+        </is>
+      </c>
       <c r="G2" s="4" t="n"/>
       <c r="H2" s="4" t="inlineStr">
         <is>
+          <t>https://openalex.org/works?...</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
           <t>3 of 5</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>First version; test paper 4 missed — no 'reduced working hours' in string</t>
+      <c r="J2" s="4" t="n"/>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>First version; test paper 4 missed — no abstract in OpenAlex, title-only match failed</t>
         </is>
       </c>
     </row>
@@ -637,12 +659,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
@@ -654,19 +676,19 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Round 1 (ta = title/abstract): include / exclude / unsure. Round 2 (ft = full text): include / exclude / not retrievable — a reason is required for every full-text exclusion.</t>
+          <t>Missing abstract? Open the DOI link and copy it from the publisher page; record the source (OpenAlex / Crossref / publisher page / open-access version). Round 1 (ta): include / exclude / unsure. Round 2 (ft): include / exclude / not retrievable — a reason is required for every full-text exclusion.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>UT (WoS ID)</t>
+          <t>OpenAlex ID</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Authors</t>
+          <t>DOI</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -686,12 +708,12 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>DOI</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>abstract_source</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -730,12 +752,15 @@
   <mergeCells count="1">
     <mergeCell ref="A1:M1"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="H3:H2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"include,exclude,unsure"</formula1>
     </dataValidation>
     <dataValidation sqref="J3:J2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"include,exclude,not retrievable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G3:G2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"OpenAlex,Crossref,publisher page,open-access version"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -864,17 +889,17 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>English-language journal articles in Web of Science only</t>
+          <t>Title-and-abstract search in OpenAlex; about a third of hits without abstract</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Trial reports by campaigning organisations and German-language studies missing</t>
+          <t>Recall loss for recent closed-access articles of large publishers</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Scope of a term paper; reported explicitly; key reports discussed separately</t>
+          <t>No open alternative; compensated by compulsory snowballing; share reported</t>
         </is>
       </c>
     </row>

</xml_diff>